<commit_message>
Add analysis by task type
</commit_message>
<xml_diff>
--- a/1_input_prompts/20250504_Prompts.xlsx
+++ b/1_input_prompts/20250504_Prompts.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10402"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bhabalaj/Repositories/UNEP/unep-life-cycle-assessment-ml-paper-evaluation/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\projects\unep-life-cycle-assessment-ml-paper-evaluation\1_input_prompts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0401C33E-BEED-C84A-8C10-8A6A36B495BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F259F15-841D-4AE6-92D8-25E986EA4C30}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="23240" windowHeight="13880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="13872" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="prompt_list" sheetId="5" r:id="rId1"/>
@@ -45,21 +45,12 @@
     <author>tc={06172AAA-029A-4A72-AE0E-2AC15896B46F}</author>
   </authors>
   <commentList>
-    <comment ref="C1" authorId="0" shapeId="0" xr:uid="{06172AAA-029A-4A72-AE0E-2AC15896B46F}">
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{06172AAA-029A-4A72-AE0E-2AC15896B46F}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     This is based on the list of filters on Hugging Face when searching for models and datasets</t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -74,19 +65,10 @@
   <commentList>
     <comment ref="E3" authorId="0" shapeId="0" xr:uid="{B1E4C3CC-781B-4A61-8340-B3A53EB2CF0F}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Very generic answer. Starts talking about EIA, which is not in the scope of the question which specifies this is a LCA scenario</t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -105,90 +87,45 @@
   <commentList>
     <comment ref="C1" authorId="0" shapeId="0" xr:uid="{28A8AFCD-029C-4A8E-B180-6B63A99BDF07}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     These prompts are representative of a casual chat with an AI model. If you want to automate a task repeatedly, the instructions to the model would be much more precise and carefully structured. 
 Here is an example from the Parakeet paper: https://github.com/amazon-science/carbon-assessment-with-ml/blob/main/parakeet/src/prompts.py#L113 </t>
-        </r>
       </text>
     </comment>
     <comment ref="C3" authorId="1" shapeId="0" xr:uid="{7D1644DC-076B-41B2-B167-10921F262697}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     This prompt is very difficult to evaluate. If 100 humans were given the task of writing the literature review, they will come up with completely different versions. If 100 experts were to review the results, the variance of their evaluation will be high. </t>
-        </r>
       </text>
     </comment>
     <comment ref="B6" authorId="2" shapeId="0" xr:uid="{8C53B1FA-3BD8-4236-BC3B-EB58811E0A13}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t xml:space="preserve">[Threaded comment]
+        <t xml:space="preserve">[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Citation ability is entirely dependent on the giving the model access to sufficient resources:
 1. Will it be given access to the internet?
 2. Will the "reason" button be toggled? </t>
-        </r>
       </text>
     </comment>
     <comment ref="C8" authorId="3" shapeId="0" xr:uid="{C20EC0BD-2878-4504-BDEC-0C4CB880759D}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Todo: create an excel that can be input, and figure a way to pass this programmatically to the model</t>
-        </r>
       </text>
     </comment>
     <comment ref="C9" authorId="4" shapeId="0" xr:uid="{AE9B5153-A15E-40E5-A643-B73A1ED6E550}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Aptos Narrow"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Todo, choose a paper</t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -196,7 +133,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="150">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="283" uniqueCount="151">
   <si>
     <t>LCA stage</t>
   </si>
@@ -1186,6 +1123,9 @@
   </si>
   <si>
     <t>Extra_remarks</t>
+  </si>
+  <si>
+    <t>ID</t>
   </si>
 </sst>
 </file>
@@ -1756,7 +1696,7 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="C1" dT="2025-04-28T14:03:22.59" personId="{BFC6DB03-0879-42FD-9DA1-54534F1A8D8C}" id="{06172AAA-029A-4A72-AE0E-2AC15896B46F}">
+  <threadedComment ref="D1" dT="2025-04-28T14:03:22.59" personId="{BFC6DB03-0879-42FD-9DA1-54534F1A8D8C}" id="{06172AAA-029A-4A72-AE0E-2AC15896B46F}">
     <text>This is based on the list of filters on Hugging Face when searching for models and datasets</text>
   </threadedComment>
 </ThreadedComments>
@@ -1801,435 +1741,510 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{14947F5A-EF3E-4553-A69B-A4AC7AC65870}">
-  <dimension ref="A1:G25"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:H25"/>
+  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="3" max="3" width="13.83203125" style="5" customWidth="1"/>
-    <col min="4" max="4" width="73.83203125" customWidth="1"/>
+    <col min="4" max="4" width="13.83984375" style="5" customWidth="1"/>
+    <col min="5" max="5" width="73.83984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B1" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="C1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="D1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="117.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+    <row r="2" spans="1:8" ht="117.55" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="C2" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="D2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="E2" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="192" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
+    <row r="3" spans="1:8" ht="172.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="D3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>13</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="192" x14ac:dyDescent="0.2">
-      <c r="A4" t="s">
+    <row r="4" spans="1:8" ht="172.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>6</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="C4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="D4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="E4" t="s">
+      <c r="F4" t="s">
         <v>16</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="128" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
+    <row r="5" spans="1:8" ht="115.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="C5" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="E5" t="s">
+      <c r="F5" t="s">
         <v>19</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="350" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
+    <row r="6" spans="1:8" ht="316.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="C6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="D6" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>10</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="48" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
-        <v>23</v>
+    <row r="7" spans="1:8" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A7">
+        <v>6</v>
       </c>
       <c r="B7" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C7" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>25</v>
       </c>
-      <c r="E7" t="s">
+      <c r="F7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="272" x14ac:dyDescent="0.2">
-      <c r="A8" s="5" t="s">
-        <v>23</v>
+    <row r="8" spans="1:8" ht="259.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A8">
+        <v>7</v>
       </c>
       <c r="B8" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C8" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="160" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
+    <row r="9" spans="1:8" ht="144" x14ac:dyDescent="0.55000000000000004">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>29</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="D9" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="192" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
-        <v>6</v>
+    <row r="10" spans="1:8" ht="187.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A10">
+        <v>9</v>
       </c>
       <c r="B10" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" t="s">
+        <v>6</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="288" x14ac:dyDescent="0.2">
-      <c r="A11" s="5" t="s">
-        <v>23</v>
+    <row r="11" spans="1:8" ht="273.60000000000002" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11">
+        <v>10</v>
       </c>
       <c r="B11" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="H11" s="5" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="128" x14ac:dyDescent="0.2">
-      <c r="A12" s="5" t="s">
+    <row r="12" spans="1:8" ht="129.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12">
+        <v>11</v>
+      </c>
+      <c r="B12" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="E12" s="5" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="48" x14ac:dyDescent="0.2">
-      <c r="A13" s="5" t="s">
+    <row r="13" spans="1:8" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A13">
+        <v>12</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="C13" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="48" x14ac:dyDescent="0.2">
-      <c r="A14" s="5" t="s">
+    <row r="14" spans="1:8" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A14">
+        <v>13</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E14" t="s">
+      <c r="F14" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="48" x14ac:dyDescent="0.2">
-      <c r="A15" s="5" t="s">
+    <row r="15" spans="1:8" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A15">
+        <v>14</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E15" t="s">
+      <c r="F15" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A16" s="5" t="s">
+    <row r="16" spans="1:8" ht="409.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A16">
+        <v>15</v>
+      </c>
+      <c r="B16" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="D16" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A17" s="5" t="s">
+    <row r="17" spans="1:6" ht="374.4" x14ac:dyDescent="0.55000000000000004">
+      <c r="A17">
+        <v>16</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="D17" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>49</v>
       </c>
-      <c r="E17" t="s">
+      <c r="F17" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="409.6" x14ac:dyDescent="0.2">
-      <c r="A18" s="5" t="s">
+    <row r="18" spans="1:6" ht="409.5" x14ac:dyDescent="0.55000000000000004">
+      <c r="A18">
+        <v>17</v>
+      </c>
+      <c r="B18" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="C18" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="5" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="224" x14ac:dyDescent="0.2">
-      <c r="A19" s="5" t="s">
+    <row r="19" spans="1:6" ht="201.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19">
+        <v>18</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="D19" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="5" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+    <row r="20" spans="1:6" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
         <v>6</v>
       </c>
-      <c r="B20" s="5" t="s">
+      <c r="C20" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="D20" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="E20" s="11" t="s">
         <v>54</v>
       </c>
-      <c r="E20" t="s">
+      <c r="F20" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+    <row r="21" spans="1:6" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
         <v>6</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="D21" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D21" s="12" t="s">
+      <c r="E21" s="12" t="s">
         <v>56</v>
       </c>
-      <c r="E21" t="s">
+      <c r="F21" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+    <row r="22" spans="1:6" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A22">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
         <v>6</v>
       </c>
-      <c r="B22" s="5" t="s">
+      <c r="C22" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="D22" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="E22" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E22" t="s">
+      <c r="F22" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="64" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
-        <v>6</v>
+    <row r="23" spans="1:6" ht="57.6" x14ac:dyDescent="0.55000000000000004">
+      <c r="A23">
+        <v>22</v>
       </c>
       <c r="B23" t="s">
         <v>6</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" t="s">
+        <v>6</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="E23" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="E23" t="s">
+      <c r="F23" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="48" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+    <row r="24" spans="1:6" ht="43.2" x14ac:dyDescent="0.55000000000000004">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
         <v>6</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>38</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="D24" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="E24" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="E24" t="s">
+      <c r="F24" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="32" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+    <row r="25" spans="1:6" ht="28.8" x14ac:dyDescent="0.55000000000000004">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
         <v>6</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>64</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="D25" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E25" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="E25" t="s">
+      <c r="F25" t="s">
         <v>66</v>
       </c>
     </row>
@@ -2243,49 +2258,49 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFD02E40-FF3A-499A-B02D-2B2A7584557C}">
   <dimension ref="A2:A10"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>67</v>
       </c>
@@ -2301,14 +2316,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{618D7821-FBDB-45D5-9AFD-8501E7E29E27}">
   <dimension ref="A1:D21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="31.5" customWidth="1"/>
-    <col min="3" max="3" width="23.1640625" customWidth="1"/>
-    <col min="4" max="4" width="24.1640625" customWidth="1"/>
+    <col min="1" max="1" width="31.47265625" customWidth="1"/>
+    <col min="3" max="3" width="23.15625" customWidth="1"/>
+    <col min="4" max="4" width="24.15625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="C1" s="8" t="s">
         <v>68</v>
       </c>
@@ -2316,7 +2331,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="28" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="23.4" x14ac:dyDescent="0.55000000000000004">
       <c r="C2" s="10" t="s">
         <v>70</v>
       </c>
@@ -2324,7 +2339,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>72</v>
       </c>
@@ -2335,7 +2350,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>73</v>
       </c>
@@ -2346,7 +2361,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>74</v>
       </c>
@@ -2357,7 +2372,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>75</v>
       </c>
@@ -2368,7 +2383,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>64</v>
       </c>
@@ -2379,7 +2394,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>77</v>
       </c>
@@ -2390,7 +2405,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>78</v>
       </c>
@@ -2401,7 +2416,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>79</v>
       </c>
@@ -2412,7 +2427,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>80</v>
       </c>
@@ -2423,7 +2438,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>81</v>
       </c>
@@ -2434,7 +2449,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>82</v>
       </c>
@@ -2445,7 +2460,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>83</v>
       </c>
@@ -2456,7 +2471,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>36</v>
       </c>
@@ -2467,7 +2482,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>84</v>
       </c>
@@ -2478,7 +2493,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>85</v>
       </c>
@@ -2489,7 +2504,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
         <v>86</v>
       </c>
@@ -2500,7 +2515,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="32" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
         <v>87</v>
       </c>
@@ -2511,7 +2526,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
         <v>88</v>
       </c>
@@ -2522,7 +2537,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
         <v>89</v>
       </c>
@@ -2544,21 +2559,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A2:P8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="28.5" customWidth="1"/>
-    <col min="2" max="2" width="87.5" customWidth="1"/>
-    <col min="3" max="4" width="21.33203125" customWidth="1"/>
-    <col min="5" max="6" width="52.1640625" customWidth="1"/>
-    <col min="7" max="8" width="33.5" customWidth="1"/>
-    <col min="9" max="10" width="24.83203125" customWidth="1"/>
-    <col min="11" max="12" width="44.5" customWidth="1"/>
-    <col min="13" max="14" width="22.33203125" customWidth="1"/>
-    <col min="15" max="15" width="21.83203125" customWidth="1"/>
-    <col min="16" max="16" width="66.33203125" customWidth="1"/>
+    <col min="1" max="1" width="28.47265625" customWidth="1"/>
+    <col min="2" max="2" width="87.47265625" customWidth="1"/>
+    <col min="3" max="4" width="21.3125" customWidth="1"/>
+    <col min="5" max="6" width="52.15625" customWidth="1"/>
+    <col min="7" max="8" width="33.47265625" customWidth="1"/>
+    <col min="9" max="10" width="24.83984375" customWidth="1"/>
+    <col min="11" max="12" width="44.47265625" customWidth="1"/>
+    <col min="13" max="14" width="22.3125" customWidth="1"/>
+    <col min="15" max="15" width="21.83984375" customWidth="1"/>
+    <col min="16" max="16" width="66.3125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:16" ht="21.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>90</v>
       </c>
@@ -2608,7 +2623,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="234.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:16" ht="234.75" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="2" t="s">
         <v>23</v>
       </c>
@@ -2632,7 +2647,7 @@
       </c>
       <c r="L3" s="5"/>
     </row>
-    <row r="4" spans="1:16" ht="136.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:16" ht="136.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>110</v>
       </c>
@@ -2644,7 +2659,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="188.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:16" ht="188.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>113</v>
       </c>
@@ -2665,7 +2680,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="6" spans="1:16" ht="80.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:16" ht="80.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>113</v>
       </c>
@@ -2683,7 +2698,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="7" spans="1:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:16" ht="34.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>76</v>
       </c>
@@ -2701,7 +2716,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="8" spans="1:16" ht="149.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:16" ht="149.25" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -2728,7 +2743,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF9400C8-20FE-4648-BD9A-7ECDA9196870}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2738,17 +2753,17 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A1DB77A-BE06-496A-8AB3-8005711EB4C0}">
   <dimension ref="A1:F13"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.83984375" defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="15.6640625" style="5" customWidth="1"/>
-    <col min="2" max="2" width="31.83203125" customWidth="1"/>
+    <col min="1" max="1" width="15.68359375" style="5" customWidth="1"/>
+    <col min="2" max="2" width="31.83984375" customWidth="1"/>
     <col min="3" max="3" width="83" customWidth="1"/>
-    <col min="4" max="4" width="8.83203125" customWidth="1"/>
-    <col min="5" max="5" width="37.83203125" customWidth="1"/>
-    <col min="6" max="6" width="32.6640625" customWidth="1"/>
+    <col min="4" max="4" width="8.83984375" customWidth="1"/>
+    <col min="5" max="5" width="37.83984375" customWidth="1"/>
+    <col min="6" max="6" width="32.68359375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -2768,7 +2783,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="191" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="191.05" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="5" t="s">
         <v>23</v>
       </c>
@@ -2782,7 +2797,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="128.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="128.5" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="5" t="s">
         <v>23</v>
       </c>
@@ -2796,7 +2811,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5" t="s">
         <v>38</v>
       </c>
@@ -2813,13 +2828,13 @@
         <v>133</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.55000000000000004">
       <c r="B5" s="5"/>
       <c r="C5" s="5"/>
       <c r="D5" s="5"/>
       <c r="F5" s="5"/>
     </row>
-    <row r="6" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" s="5" t="s">
         <v>38</v>
       </c>
@@ -2833,7 +2848,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" s="5" t="s">
         <v>38</v>
       </c>
@@ -2850,7 +2865,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="5" t="s">
         <v>6</v>
       </c>
@@ -2864,7 +2879,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="5" t="s">
         <v>36</v>
       </c>
@@ -2878,7 +2893,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" ht="409.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="5" t="s">
         <v>142</v>
       </c>
@@ -2892,7 +2907,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" ht="409.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" s="5" t="s">
         <v>142</v>
       </c>
@@ -2909,7 +2924,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" ht="409.5" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" s="5" t="s">
         <v>142</v>
       </c>
@@ -2926,7 +2941,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" ht="43.2" x14ac:dyDescent="0.55000000000000004">
       <c r="B13" t="s">
         <v>147</v>
       </c>
@@ -2944,33 +2959,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4ace1cb2-4842-4f43-9eb1-c2ca1b56feb0">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d47708fc-08f7-4182-878a-2b4f8b9059a7" xsi:nil="true"/>
-    <Owner xmlns="4ace1cb2-4842-4f43-9eb1-c2ca1b56feb0">
-      <UserInfo>
-        <DisplayName/>
-        <AccountId xsi:nil="true"/>
-        <AccountType/>
-      </UserInfo>
-    </Owner>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101005886909632557E4DA4D69A2DAD165CFA" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="afeba9c07da46cf129f9ec78106790e3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4ace1cb2-4842-4f43-9eb1-c2ca1b56feb0" xmlns:ns3="d47708fc-08f7-4182-878a-2b4f8b9059a7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="861c48f6a3e7df37ff7c677cf88d1ebc" ns2:_="" ns3:_="">
     <xsd:import namespace="4ace1cb2-4842-4f43-9eb1-c2ca1b56feb0"/>
@@ -3191,10 +3179,48 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4ace1cb2-4842-4f43-9eb1-c2ca1b56feb0">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d47708fc-08f7-4182-878a-2b4f8b9059a7" xsi:nil="true"/>
+    <Owner xmlns="4ace1cb2-4842-4f43-9eb1-c2ca1b56feb0">
+      <UserInfo>
+        <DisplayName/>
+        <AccountId xsi:nil="true"/>
+        <AccountType/>
+      </UserInfo>
+    </Owner>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50C8ECDD-ABAF-4B7F-9D45-81F0F77C9D8E}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12E72801-A8A9-46FF-95B4-BCF039A26605}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="4ace1cb2-4842-4f43-9eb1-c2ca1b56feb0"/>
+    <ds:schemaRef ds:uri="d47708fc-08f7-4182-878a-2b4f8b9059a7"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -3211,20 +3237,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{12E72801-A8A9-46FF-95B4-BCF039A26605}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50C8ECDD-ABAF-4B7F-9D45-81F0F77C9D8E}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="4ace1cb2-4842-4f43-9eb1-c2ca1b56feb0"/>
-    <ds:schemaRef ds:uri="d47708fc-08f7-4182-878a-2b4f8b9059a7"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>